<commit_message>
Push outputs from CI/CD (2026-09-28 18:51:59)
</commit_message>
<xml_diff>
--- a/production/extension-CHECKED/Manufacturing/Assembly/ZSWatch-Extension-bom.xlsx
+++ b/production/extension-CHECKED/Manufacturing/Assembly/ZSWatch-Extension-bom.xlsx
@@ -746,10 +746,10 @@
     <t>Created:</t>
   </si>
   <si>
-    <t>2026-02-20 14:45:12</t>
-  </si>
-  <si>
-    <t>KiCost® v1.1.20 + KiBot v1.8.5</t>
+    <t>2026-09-28 18:56:30</t>
+  </si>
+  <si>
+    <t>KiCost® v1.1.21 + KiBot v1.9.1</t>
   </si>
   <si>
     <t>Columns colors</t>
@@ -2837,7 +2837,7 @@
     <row r="47" spans="10:10" ht="30" hidden="1" customHeight="1">
       <c r="J47" t="str">
         <f t="array" ref="J47:J63">IF(ISNUMBER(J10:J26)*(J10:J26&gt;=L10:L26)*(N10:N26&lt;&gt;""),N10:N26&amp;"|"&amp;TEXT(ROUNDUP(J10:J26/IF(ISNUMBER(L10:L26),L10:L26,1),0)*L10:L26,"##0")&amp;"|"&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(IF(PURCHASE_DESCRIPTION&lt;&gt;"",PURCHASE_DESCRIPTION&amp;":","")&amp;A10:A26,"|",";")," ","_"),"
-","_")&amp;CHAR(10),"")</f>
+","_")&amp;CHAR(13),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>